<commit_message>
Add points for aa59tfi9hkmjec05olroia13o_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/aa59tfi9hkmjec05olroia13o_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/aa59tfi9hkmjec05olroia13o_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG23"/>
+  <dimension ref="A1:BG32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -819,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -850,7 +850,7 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS2" t="n">
         <v>0</v>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="BG2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -955,14 +955,18 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>23</v>
-      </c>
-      <c r="O3" t="inlineStr"/>
+        <v>94</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -970,10 +974,16 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>23</v>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+        <v>71.2</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>22.8</v>
+      </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -994,10 +1004,10 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF3" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1008,45 +1018,45 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.32378458</v>
+        <v>0.72893747</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>+0.16</t>
+          <t>+0.33</t>
         </is>
       </c>
       <c r="AK3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS3" t="n">
         <v>5</v>
       </c>
-      <c r="AL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>23</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>2</v>
-      </c>
       <c r="AT3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV3" t="n">
         <v>0</v>
@@ -1078,13 +1088,13 @@
         </is>
       </c>
       <c r="BE3" t="n">
+        <v>8</v>
+      </c>
+      <c r="BF3" t="n">
         <v>3</v>
       </c>
-      <c r="BF3" t="n">
-        <v>0</v>
-      </c>
       <c r="BG3" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4">
@@ -1128,10 +1138,12 @@
           <t>d3dv3vc71981v5oems59892sq</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
@@ -1142,14 +1154,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1157,7 +1169,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1181,13 +1193,13 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF4" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -1195,21 +1207,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.22435034</v>
+        <v>-0.1750366699999999</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>+0.06</t>
+          <t>-0.57</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1221,10 +1233,10 @@
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS4" t="n">
         <v>1</v>
@@ -1233,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="AU4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV4" t="n">
         <v>0</v>
@@ -1265,13 +1277,13 @@
         </is>
       </c>
       <c r="BE4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BG4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5">
@@ -1315,10 +1327,12 @@
           <t>cionsifzpx5rhc8es29wv6i95</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -1329,14 +1343,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1344,7 +1358,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1368,13 +1382,13 @@
         <v>1</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1382,37 +1396,37 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.36522543</v>
+        <v>0.5215941299999999</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>+0.20</t>
+          <t>+0.12</t>
         </is>
       </c>
       <c r="AK5" t="n">
+        <v>11</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>82</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR5" t="n">
         <v>4</v>
       </c>
-      <c r="AL5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>23</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>1</v>
-      </c>
       <c r="AS5" t="n">
         <v>0</v>
       </c>
@@ -1423,7 +1437,7 @@
         <v>0</v>
       </c>
       <c r="AV5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -1451,7 +1465,7 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG5" t="n">
         <v>0</v>
@@ -1512,14 +1526,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1527,7 +1541,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1551,10 +1565,10 @@
         <v>1</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG6" t="n">
         <v>1</v>
@@ -1565,21 +1579,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.09930234999999998</v>
+        <v>0.1247456699999999</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.06</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1588,19 +1602,19 @@
         <v>0</v>
       </c>
       <c r="AP6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ6" t="n">
         <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AS6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU6" t="n">
         <v>0</v>
@@ -1612,7 +1626,7 @@
         <v>0</v>
       </c>
       <c r="AX6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY6" t="n">
         <v>0</v>
@@ -1634,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="BF6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG6" t="n">
         <v>0</v>
@@ -1695,14 +1709,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1710,7 +1724,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1734,10 +1748,10 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF7" t="n">
-        <v>-0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG7" t="n">
         <v>1</v>
@@ -1748,21 +1762,21 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.06043170999999999</v>
+        <v>0.3938758199999999</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.00</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1774,19 +1788,19 @@
         <v>0</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AT7" t="n">
         <v>0</v>
       </c>
       <c r="AU7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV7" t="n">
         <v>0</v>
@@ -1817,7 +1831,7 @@
         <v>0</v>
       </c>
       <c r="BF7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG7" t="n">
         <v>0</v>
@@ -1864,10 +1878,12 @@
           <t>b3974hgsmyff5xtq7qf1onhlh</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -1878,14 +1894,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1893,7 +1909,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1923,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="AG8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
@@ -1931,21 +1947,21 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>-0.29149639</v>
+        <v>-0.30964699</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.46</t>
+          <t>-0.71</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -2065,14 +2081,18 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>23</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
+        <v>94</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2080,10 +2100,16 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>23</v>
-      </c>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+        <v>82.7</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>11.3</v>
+      </c>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
@@ -2104,10 +2130,10 @@
         <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF9" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG9" t="n">
         <v>1</v>
@@ -2118,11 +2144,11 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>1.40314984</v>
+        <v>1.50283485</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+1.24</t>
+          <t>+1.10</t>
         </is>
       </c>
       <c r="AK9" t="n">
@@ -2132,7 +2158,7 @@
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN9" t="n">
         <v>1</v>
@@ -2141,22 +2167,22 @@
         <v>0</v>
       </c>
       <c r="AP9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ9" t="n">
         <v>0</v>
       </c>
       <c r="AR9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS9" t="n">
         <v>0</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2188,13 +2214,13 @@
         </is>
       </c>
       <c r="BE9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BF9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -2252,14 +2278,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2267,7 +2293,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2291,7 +2317,7 @@
         <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
@@ -2305,21 +2331,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.20613131</v>
+        <v>0.71481748</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.04</t>
+          <t>+0.32</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2381,7 +2407,7 @@
         <v>0</v>
       </c>
       <c r="BG10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -2439,14 +2465,18 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>23</v>
-      </c>
-      <c r="O11" t="inlineStr"/>
+        <v>94</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2454,10 +2484,16 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>23</v>
-      </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+        <v>82.7</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>11.3</v>
+      </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -2478,10 +2514,10 @@
         <v>1</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF11" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG11" t="n">
         <v>1</v>
@@ -2492,21 +2528,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.2749883200000001</v>
+        <v>0.71876092</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.11</t>
+          <t>+0.32</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2515,22 +2551,22 @@
         <v>0</v>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ11" t="n">
         <v>0</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT11" t="n">
         <v>0</v>
       </c>
       <c r="AU11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV11" t="n">
         <v>0</v>
@@ -2562,13 +2598,13 @@
         </is>
       </c>
       <c r="BE11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BF11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -2612,10 +2648,12 @@
           <t>6psklvi66inwws7buzf16yjft</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -2626,14 +2664,14 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2641,7 +2679,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2665,13 +2703,13 @@
         <v>1</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -2679,21 +2717,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>1.01284193</v>
+        <v>1.37656541</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+0.85</t>
+          <t>+0.98</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2705,10 +2743,10 @@
         <v>1</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
@@ -2717,7 +2755,7 @@
         <v>0</v>
       </c>
       <c r="AU12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2748,7 +2786,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2762,37 +2800,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>L. Mpasi</t>
+          <t>Nélson Semedo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>9s90f4r3095h8mefzmpuut51x</t>
+          <t>3fhoof7n4sjaizvotcmypb9at</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2801,11 +2839,15 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>71</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N13" t="n">
@@ -2813,14 +2855,14 @@
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="Q13" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S13" t="n">
@@ -2836,35 +2878,47 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Nélson Semedo</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>-0.02146554000000005</v>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>-0.42</t>
+        </is>
+      </c>
+      <c r="AK13" t="n">
+        <v>25</v>
+      </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="AM13" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2876,13 +2930,13 @@
         <v>0</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR13" t="n">
         <v>0</v>
       </c>
       <c r="AS13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT13" t="n">
         <v>0</v>
@@ -2897,7 +2951,7 @@
         <v>0</v>
       </c>
       <c r="AX13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY13" t="n">
         <v>0</v>
@@ -2919,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="BF13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG13" t="n">
         <v>0</v>
@@ -2933,37 +2987,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A. Wan-Bissaka</t>
+          <t>Gonçalo Ramos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2</t>
+          <t xml:space="preserve"> 9</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>e1t5rgvs2hwnldts6vn8agzc9</t>
+          <t>9v4l7ic3ve6d22c0gs9p1oe3u</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -2972,33 +3026,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>82</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>23</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="Q14" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>RWB</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>23</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+        <v>0.7</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>11.3</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -3007,47 +3075,47 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="AD14" t="n">
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0.2</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>A. Wan-Bissaka</t>
+          <t>Gonçalo Ramos</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.11205196</v>
+        <v>0.01042592</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="AL14" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="AM14" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3065,13 +3133,13 @@
         <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
         <v>0</v>
       </c>
       <c r="AU14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV14" t="n">
         <v>0</v>
@@ -3116,37 +3184,37 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A. Masuaku</t>
+          <t>Rafael Leão</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 26</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>55bgi895g03zhc7vdh7e7yvv9</t>
+          <t>11o903vztwpnmvgrinn208qnd</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3155,33 +3223,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>71</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N15" t="n">
         <v>23</v>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>LM</t>
+        </is>
+      </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="Q15" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LWB</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>23</v>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+        <v>11.7</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>LM</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>11.3</v>
+      </c>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
@@ -3190,47 +3272,47 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="AD15" t="n">
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>A. Masuaku</t>
+          <t>Rafael Leão</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.06312887999999997</v>
+        <v>0.20095632</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="AL15" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="AM15" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3239,16 +3321,16 @@
         <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
@@ -3280,7 +3362,11 @@
       <c r="BC15" t="n">
         <v>0</v>
       </c>
-      <c r="BD15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
       <c r="BE15" t="n">
         <v>0</v>
       </c>
@@ -3288,7 +3374,7 @@
         <v>2</v>
       </c>
       <c r="BG15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3299,37 +3385,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>S. Kapuadi</t>
+          <t>Francisco Conceição</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3</t>
+          <t xml:space="preserve"> 26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LCB(3)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>c0arcrn5kpsofa1r53m1dhqp6</t>
+          <t>2x44f29a52v8kpkkjsuiiywdm</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3338,33 +3424,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>45</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>23</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
+        <v>49</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="Q16" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LCB(3)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>23</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+        <v>37.7</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>11.3</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -3373,12 +3473,12 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+          <t>8gxg8f7p9299jbrz30u8bsc7g</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="AD16" t="n">
@@ -3388,32 +3488,32 @@
         <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>S. Kapuadi</t>
+          <t>Francisco Conceição</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>-0.18277026</v>
+        <v>0.9267406599999999</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.35</t>
+          <t>+0.53</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="AM16" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3422,22 +3522,22 @@
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT16" t="n">
         <v>0</v>
       </c>
       <c r="AU16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV16" t="n">
         <v>0</v>
@@ -3468,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BG16" t="n">
         <v>0</v>
@@ -3487,17 +3587,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A. Tuanzebe</t>
+          <t>L. Mpasi</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CB(3)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3507,12 +3607,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>cr74l0rwvkf4yck0go4esw44p</t>
+          <t>9s90f4r3095h8mefzmpuut51x</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3529,22 +3629,22 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>CB(3)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3565,38 +3665,26 @@
         </is>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE17" t="n">
         <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
         <v>1</v>
       </c>
-      <c r="AH17" t="inlineStr">
-        <is>
-          <t>A. Tuanzebe</t>
-        </is>
-      </c>
-      <c r="AI17" t="n">
-        <v>-0.26391865</v>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>-0.43</t>
-        </is>
-      </c>
-      <c r="AK17" t="n">
-        <v>19</v>
-      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="n">
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3611,10 +3699,10 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
@@ -3670,17 +3758,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>C. Mbemba</t>
+          <t>A. Wan-Bissaka</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 22</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RCB(3)</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3690,18 +3778,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>bb5eekaj9i0dbckrkb629qg2d</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>e1t5rgvs2hwnldts6vn8agzc9</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
@@ -3712,22 +3802,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>RCB(3)</t>
+          <t>RWB</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3748,7 +3838,7 @@
         </is>
       </c>
       <c r="AD18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE18" t="n">
         <v>1</v>
@@ -3757,19 +3847,19 @@
         <v>-0.2</v>
       </c>
       <c r="AG18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>C. Mbemba</t>
+          <t>A. Wan-Bissaka</t>
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>0.13999836</v>
+        <v>0.6280125099999999</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>+0.23</t>
         </is>
       </c>
       <c r="AK18" t="n">
@@ -3779,7 +3869,7 @@
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3791,19 +3881,19 @@
         <v>0</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AS18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AT18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV18" t="n">
         <v>0</v>
@@ -3834,7 +3924,7 @@
         <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BG18" t="n">
         <v>0</v>
@@ -3853,17 +3943,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>N. Mukau</t>
+          <t>A. Masuaku</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3873,18 +3963,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>9ov7tj31hixo7xp0tfffuhpn8</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>55bgi895g03zhc7vdh7e7yvv9</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -3895,22 +3987,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3931,62 +4023,62 @@
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE19" t="n">
         <v>1</v>
       </c>
       <c r="AF19" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>N. Mukau</t>
+          <t>A. Masuaku</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.0179668</v>
+        <v>0.9733951299999999</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>+0.58</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>23</v>
+        <v>74</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
       </c>
       <c r="AO19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AR19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4017,7 +4109,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4036,17 +4128,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S. Moutoussamy</t>
+          <t>S. Kapuadi</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8</t>
+          <t xml:space="preserve"> 3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4056,12 +4148,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>cg1j982govx2perwr3rv33t1x</t>
+          <t>c0arcrn5kpsofa1r53m1dhqp6</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -4078,22 +4170,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4114,38 +4206,38 @@
         </is>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE20" t="n">
         <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG20" t="n">
         <v>1</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>S. Moutoussamy</t>
+          <t>S. Kapuadi</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>-0.009355050000000004</v>
+        <v>0.32302981</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4154,7 +4246,7 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
         <v>0</v>
@@ -4163,13 +4255,13 @@
         <v>1</v>
       </c>
       <c r="AS20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT20" t="n">
         <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV20" t="n">
         <v>0</v>
@@ -4200,7 +4292,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4219,17 +4311,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C. Bakambu</t>
+          <t>A. Tuanzebe</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LCF(2)</t>
+          <t>CB(3)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4239,12 +4331,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>a68fosxpgtyxj64ex9f6nget</t>
+          <t>cr74l0rwvkf4yck0go4esw44p</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4261,22 +4353,22 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>LCF(2)</t>
+          <t>CB(3)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4297,38 +4389,38 @@
         </is>
       </c>
       <c r="AD21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE21" t="n">
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>C. Bakambu</t>
+          <t>A. Tuanzebe</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.38032736</v>
+        <v>0.1094796799999999</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.22</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4340,19 +4432,19 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV21" t="n">
         <v>0</v>
@@ -4383,7 +4475,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -4402,17 +4494,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Y. Wissa</t>
+          <t>C. Mbemba</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 22</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RCF(2)</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4422,12 +4514,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>bxjc2heo4ve54cyvw98qcck45</t>
+          <t>bb5eekaj9i0dbckrkb629qg2d</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4444,22 +4536,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>RCF(2)</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4480,38 +4572,38 @@
         </is>
       </c>
       <c r="AD22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE22" t="n">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>Y. Wissa</t>
+          <t>C. Mbemba</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>-0.02682477</v>
+        <v>0.27335769</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4520,31 +4612,31 @@
         <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ22" t="n">
         <v>0</v>
       </c>
       <c r="AR22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AT22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW22" t="n">
         <v>0</v>
       </c>
       <c r="AX22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY22" t="n">
         <v>0</v>
@@ -4566,7 +4658,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -4585,17 +4677,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>E. Kayembe</t>
+          <t>N. Mukau</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 25</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4605,18 +4697,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>dgrk1cgbyk03p3e32nj4yugru</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>9ov7tj31hixo7xp0tfffuhpn8</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -4627,22 +4721,22 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4663,7 +4757,7 @@
         </is>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE23" t="n">
         <v>1</v>
@@ -4672,29 +4766,29 @@
         <v>-0.05</v>
       </c>
       <c r="AG23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>E. Kayembe</t>
+          <t>N. Mukau</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.14607222</v>
+        <v>0.01435955</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4703,19 +4797,19 @@
         <v>0</v>
       </c>
       <c r="AP23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS23" t="n">
         <v>1</v>
       </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU23" t="n">
         <v>0</v>
@@ -4752,6 +4846,1687 @@
         <v>1</v>
       </c>
       <c r="BG23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>S. Moutoussamy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CM(3)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>cg1j982govx2perwr3rv33t1x</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>94</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>94</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>CM(3)</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>94</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>S. Moutoussamy</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>-0.08227408999999999</v>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>-0.48</t>
+        </is>
+      </c>
+      <c r="AK24" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>C. Bakambu</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 17</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>a68fosxpgtyxj64ex9f6nget</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>84</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>84</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>84</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>C. Bakambu</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>0.9616784899999999</v>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>+0.56</t>
+        </is>
+      </c>
+      <c r="AK25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>84</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Y. Wissa</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 20</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>RCF(2)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>bxjc2heo4ve54cyvw98qcck45</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>94</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>94</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>RCF(2)</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>94</v>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>Y. Wissa</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>1.44403839</v>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>+1.05</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>E. Kayembe</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 25</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>dgrk1cgbyk03p3e32nj4yugru</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>73</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>RCM(3)</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>73</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>RCM(3)</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>E. Kayembe</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>0.34704694</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>-0.05</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>73</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>5</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>J. Kayembe</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>4pbx40gvdmacim2n0k2qt41cl</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>74</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>20</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>94</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>20</v>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>J. Kayembe</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.17005</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>-0.23</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>17</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>74</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>N. Sadiki</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 14</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>dwnd8j9ok6ncbp69gmchw953o</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>56</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>38</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>94</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>38</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>N. Sadiki</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.1198296</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>-0.28</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>19</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>56</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>C. Pickel</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 18</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>a8ez7qv4n62b8s45pdo8u07o5</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>73</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>21</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>73</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>94</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>21</v>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>C. Pickel</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.0001422400000000018</v>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>-0.40</t>
+        </is>
+      </c>
+      <c r="AK30" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>73</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>S. Banza</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 23</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>43xutn1unln5o3gwx3cl4lo0l</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>84</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>10</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>94</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>LCF(2)</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>10</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>S. Banza</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>-0.06480321</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>-0.46</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>84</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>aa59tfi9hkmjec05olroia13o</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>G. Kalulu</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 24</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>322sju1vi12p0r9a8048hnmxh</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>84</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>10</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>94</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>10</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>dd4ko7d3muqheb54u1s9k39p3</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Congo DR</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>G. Kalulu</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>0.006495539999999994</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.39</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>84</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>94</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG32" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>